<commit_message>
start to reshape project
</commit_message>
<xml_diff>
--- a/Active June.xlsx
+++ b/Active June.xlsx
@@ -121,7 +121,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="d\-mmm"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -191,7 +191,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FFC9211E"/>
+      <color rgb="FF5983B0"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="134"/>
@@ -200,6 +200,14 @@
       <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFC9211E"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="134"/>
@@ -266,7 +274,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -332,6 +340,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -392,7 +404,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF3FAF46"/>
@@ -956,7 +968,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="17" t="s">
         <v>28</v>
       </c>
       <c r="B9" s="5" t="s">

</xml_diff>